<commit_message>
Modify functions for BondPrice and Callability for consistency reasons and add excel unit tests.
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_bonds.xlsx
+++ b/tests/workbooks/test_bonds.xlsx
@@ -8,23 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6695F9E2-73C9-4290-88B1-F38E45AEE320}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804525A8-9446-4835-9374-D51F9E284B26}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="32370" windowHeight="9360" xr2:uid="{A8952777-E146-413E-A9B0-D4A573A66C27}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabs" sheetId="1" r:id="rId1"/>
-    <sheet name="Bond" sheetId="3" r:id="rId2"/>
-    <sheet name="ZeroCouponBond" sheetId="4" r:id="rId3"/>
-    <sheet name="FixedRateBond" sheetId="5" r:id="rId4"/>
-    <sheet name="AmortizingFixedRateBond" sheetId="6" r:id="rId5"/>
-    <sheet name="AmortizingFloatingRateBond" sheetId="7" r:id="rId6"/>
-    <sheet name="FloatingRateBond" sheetId="8" r:id="rId7"/>
-    <sheet name="CmsRateBond" sheetId="9" r:id="rId8"/>
-    <sheet name="AmortizingCmsRateBond" sheetId="10" r:id="rId9"/>
-    <sheet name="CallableFixedRateBond" sheetId="13" r:id="rId10"/>
-    <sheet name="CallableZeroCouponBond" sheetId="14" r:id="rId11"/>
-    <sheet name="CPIBond" sheetId="17" r:id="rId12"/>
+    <sheet name="BondPrice" sheetId="18" r:id="rId2"/>
+    <sheet name="Bond" sheetId="3" r:id="rId3"/>
+    <sheet name="ZeroCouponBond" sheetId="4" r:id="rId4"/>
+    <sheet name="FixedRateBond" sheetId="5" r:id="rId5"/>
+    <sheet name="AmortizingFixedRateBond" sheetId="6" r:id="rId6"/>
+    <sheet name="AmortizingFloatingRateBond" sheetId="7" r:id="rId7"/>
+    <sheet name="FloatingRateBond" sheetId="8" r:id="rId8"/>
+    <sheet name="CmsRateBond" sheetId="9" r:id="rId9"/>
+    <sheet name="AmortizingCmsRateBond" sheetId="10" r:id="rId10"/>
+    <sheet name="Callability" sheetId="21" r:id="rId11"/>
+    <sheet name="CallableFixedRateBond" sheetId="13" r:id="rId12"/>
+    <sheet name="CallableZeroCouponBond" sheetId="14" r:id="rId13"/>
+    <sheet name="CPIBond" sheetId="17" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="135">
   <si>
     <t>Bond</t>
   </si>
@@ -390,6 +392,57 @@
   </si>
   <si>
     <t>BlackCallableFixedRateBondEngine</t>
+  </si>
+  <si>
+    <t>BondPrice</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>clean</t>
+  </si>
+  <si>
+    <t>qlBondPrice</t>
+  </si>
+  <si>
+    <t>qlBondPriceAmount</t>
+  </si>
+  <si>
+    <t>qlBondPriceType</t>
+  </si>
+  <si>
+    <t>qlBondPriceIsValid</t>
+  </si>
+  <si>
+    <t>Callability</t>
+  </si>
+  <si>
+    <t>price (qlBondPrice)</t>
+  </si>
+  <si>
+    <t>callability_type</t>
+  </si>
+  <si>
+    <t>put</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>qlCallability</t>
+  </si>
+  <si>
+    <t>qlCallabilityPrice</t>
+  </si>
+  <si>
+    <t>qlCallabilityDate</t>
+  </si>
+  <si>
+    <t>qlCallabilityType</t>
   </si>
 </sst>
 </file>
@@ -451,7 +504,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -554,11 +607,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -605,6 +671,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -614,9 +686,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -931,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1B31AC-6B78-4845-B599-86FA814CB2D7}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="16"/>
@@ -946,11 +1015,11 @@
       <c r="B2" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="27"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="33"/>
     </row>
     <row r="3" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="18"/>
@@ -965,18 +1034,16 @@
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="23"/>
+      <c r="B4" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="21" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>114</v>
@@ -986,7 +1053,7 @@
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="21" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>114</v>
@@ -996,7 +1063,7 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="21" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>114</v>
@@ -1006,7 +1073,7 @@
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="21" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>114</v>
@@ -1016,7 +1083,7 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="21" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" s="22" t="s">
         <v>114</v>
@@ -1026,7 +1093,7 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>114</v>
@@ -1035,8 +1102,8 @@
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="31" t="s">
-        <v>7</v>
+      <c r="B11" s="21" t="s">
+        <v>6</v>
       </c>
       <c r="C11" s="22" t="s">
         <v>114</v>
@@ -1045,28 +1112,46 @@
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="22"/>
+      <c r="B12" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>114</v>
+      </c>
       <c r="D12" s="22"/>
       <c r="E12" s="23"/>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="29" t="s">
-        <v>9</v>
+      <c r="B13" s="28" t="s">
+        <v>126</v>
       </c>
       <c r="C13" s="22"/>
       <c r="D13" s="22"/>
       <c r="E13" s="23"/>
     </row>
-    <row r="14" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="30" t="s">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+    </row>
+    <row r="16" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="25"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1078,6 +1163,929 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ABD84F-1436-4AE1-BC17-091C65B56114}">
+  <dimension ref="A1:C67"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="48.5703125" customWidth="1"/>
+    <col min="2" max="2" width="69.140625" customWidth="1"/>
+    <col min="3" max="3" width="71.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2">
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2">
+        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="3">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="34"/>
+      <c r="B6" s="3">
+        <v>102</v>
+      </c>
+      <c r="C6" s="3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="34"/>
+      <c r="B7" s="3">
+        <v>101</v>
+      </c>
+      <c r="C7" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="12">
+        <v>45665</v>
+      </c>
+      <c r="C8" s="12">
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="12">
+        <v>46030</v>
+      </c>
+      <c r="C9" s="12">
+        <v>46030</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C11" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="6">
+        <v>0</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <f>_xll.qlSchedule(B8,B9,B10,B11,B12,B13,B14,B15)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R16C2Schedule,A</v>
+      </c>
+      <c r="C16" s="3" t="str">
+        <f>_xll.qlSchedule(C8,C9,C10,C11,C12,C13,C14,C15)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R16C3Schedule,A</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6">
+        <v>2</v>
+      </c>
+      <c r="C19" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C21" s="6" t="str">
+        <f>_xll.qlCalendar("TARGET")</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="6" t="str">
+        <f>_xll.qlEuribor("3M")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R25C2Euribor,A</v>
+      </c>
+      <c r="C25" s="6" t="str">
+        <f>_xll.qlEuribor("3M")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R25C3Euribor,A</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B26" s="6" t="str">
+        <f>_xll.qlFlatForward(#REF!,0.03,"Actual360","Compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R26C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="C26" s="6" t="str">
+        <f>_xll.qlFlatForward(#REF!,0.03,"Actual360","Compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R26C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>102</v>
+      </c>
+      <c r="B27" s="3" t="str">
+        <f>_xll.qlSwapIndex(B17,B18,B19,B20,B21,B22,B23,B24,B25,B26)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R27C2SwapIndex,A</v>
+      </c>
+      <c r="C27" s="3" t="str">
+        <f>_xll.qlSwapIndex(C17,C18,C19,C20,C21,C22,C23,C24,C25,C26)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R27C3SwapIndex,A</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="2">
+        <v>45663</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B37" t="str">
+        <f>_xll.qlAmortizingCmsRateBond(B4,B5:B7,B16,B27,B28)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R37C2AmortizingCmsRateBond,A</v>
+      </c>
+      <c r="C37" t="str">
+        <f>_xll.qlAmortizingCmsRateBond(C4,C5:C7,C16,C27,C28,C29,C30,C31,C32,C33,C34,C35,C36)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R37C3AmortizingCmsRateBond,A</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="3">
+        <f>_xll.qlBondNextCouponRate(B37)</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="3">
+        <f>_xll.qlBondNextCouponRate(C37)</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" s="3">
+        <f>_xll.qlBondPreviousCouponRate(B37)</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="3">
+        <f>_xll.qlBondPreviousCouponRate(C37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" s="2">
+        <f>_xll.qlBondNextCashFlowDate(B37)</f>
+        <v>45755</v>
+      </c>
+      <c r="C40" s="2">
+        <f>_xll.qlBondNextCashFlowDate(C37)</f>
+        <v>45755</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="2">
+        <f>_xll.qlBondPreviousCashFlowDate(B37)</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="2">
+        <f>_xll.qlBondPreviousCashFlowDate(C37)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42" s="3">
+        <f>_xll.qlBondSettlementDays(B37)</f>
+        <v>2</v>
+      </c>
+      <c r="C42" s="3">
+        <f>_xll.qlBondSettlementDays(C37)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B43" s="2">
+        <f>_xll.qlBondSettlementDate(B37)</f>
+        <v>45667</v>
+      </c>
+      <c r="C43" s="2">
+        <f>_xll.qlBondSettlementDate(C37)</f>
+        <v>45667</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="3" t="b">
+        <f>_xll.qlBondIsTradable(B37)</f>
+        <v>1</v>
+      </c>
+      <c r="C44" s="3" t="b">
+        <f>_xll.qlBondIsTradable(C37)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B45" s="2">
+        <f>_xll.qlBondStartDate(B37)</f>
+        <v>45665</v>
+      </c>
+      <c r="C45" s="2">
+        <f>_xll.qlBondStartDate(C37)</f>
+        <v>45665</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46" s="2">
+        <f>_xll.qlBondMaturityDate(B37)</f>
+        <v>46030</v>
+      </c>
+      <c r="C46" s="2">
+        <f>_xll.qlBondMaturityDate(C37)</f>
+        <v>46030</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B47" s="3">
+        <f>_xll.qlBondIssueDate(B37)</f>
+        <v>0</v>
+      </c>
+      <c r="C47" s="3">
+        <f>_xll.qlBondIssueDate(C37)</f>
+        <v>45663</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B48" s="3" t="str">
+        <f>_xll.qlBondCashFlows(B37)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R48C2CashFlow,A</v>
+      </c>
+      <c r="C48" s="3" t="str">
+        <f>_xll.qlBondCashFlows(C37)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R48C3CashFlow,A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="3" t="str">
+        <f>_xll.qlBondRedemption(B37)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+    return bond.redemption()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
+    return _QuantLib.Bond_redemption(self)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
+RuntimeError: multiple redemption cash flows given
+</v>
+      </c>
+      <c r="C49" s="3" t="str">
+        <f>_xll.qlBondRedemption(C37)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+    return bond.redemption()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
+    return _QuantLib.Bond_redemption(self)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
+RuntimeError: multiple redemption cash flows given
+</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50" s="3" t="str">
+        <f>_xll.qlBondRedemptions(B37)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R50C2CashFlow,A</v>
+      </c>
+      <c r="C50" s="3" t="str">
+        <f>_xll.qlBondRedemptions(C37)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R50C3CashFlow,A</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B51" s="3" t="str">
+        <f>_xll.qlBondCalendar(B37)</f>
+        <v>TARGET</v>
+      </c>
+      <c r="C51" s="3" t="str">
+        <f>_xll.qlBondCalendar(C37)</f>
+        <v>TARGET</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B52" s="3">
+        <f>_xll.qlBondNotional(B37)</f>
+        <v>103</v>
+      </c>
+      <c r="C52" s="3">
+        <f>_xll.qlBondNotional(C37)</f>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="3">
+        <f>_xll.qlBondNotionals(B37)</f>
+        <v>103</v>
+      </c>
+      <c r="C53" s="3">
+        <f>_xll.qlBondNotionals(C37)</f>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3" t="str">
+        <f>_xll.qlFlatForward(#REF!,0.3,"actual360","compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R54C2YieldTermStructureHandle,A</v>
+      </c>
+      <c r="C54" s="3" t="str">
+        <f>_xll.qlFlatForward(#REF!,0.3,"actual360","compounded","Quarterly")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R54C3YieldTermStructureHandle,A</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" s="3" t="str">
+        <f>_xll.qlBondSetDiscountingEngine(B37,B54)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R55C2DiscountingBondEngine,A</v>
+      </c>
+      <c r="C55" s="3" t="str">
+        <f>_xll.qlBondSetDiscountingEngine(C37,C54)</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R55C3DiscountingBondEngine,A</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B56" s="10">
+        <f>_xll.qlBondCleanPrice(B37)</f>
+        <v>74.994672295319077</v>
+      </c>
+      <c r="C56" s="10">
+        <f>_xll.qlBondCleanPrice(C37)</f>
+        <v>75.244545975491022</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57" s="10">
+        <v>0.28928264971926221</v>
+      </c>
+      <c r="C57" s="10">
+        <v>0.28928264971926221</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B58" s="10">
+        <f>_xll.qlBondCleanPrice2(B37,B57,"actual360","continuous")</f>
+        <v>74.994672041966595</v>
+      </c>
+      <c r="C58" s="10">
+        <f>_xll.qlBondCleanPrice2(C37,C57,"actual360","continuous")</f>
+        <v>75.244545721623112</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B59" s="10">
+        <f>_xll.qlBondDirtyPrice(B37)</f>
+        <v>74.994672295319077</v>
+      </c>
+      <c r="C59" s="10">
+        <f>_xll.qlBondDirtyPrice(C37)</f>
+        <v>75.246212642157701</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B60" s="10">
+        <f>_xll.qlBondDirtyPrice2(B37,B57,"actual360","CONTINUOUS","annual")</f>
+        <v>74.994672041966595</v>
+      </c>
+      <c r="C60" s="10">
+        <f>_xll.qlBondDirtyPrice2(C37,C57,"actual360","CONTINUOUS","annual")</f>
+        <v>75.246212388289791</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B61" s="10" t="str">
+        <f>_xll.qlBondYield(B37,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C61" s="10">
+        <f>_xll.qlBondYield(C37,"actual360","CONTINUOUS","annual")</f>
+        <v>0.28928264793774228</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B62" s="10" t="str">
+        <f>_xll.qlBondPrice(B56,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R62C2BondPrice,A</v>
+      </c>
+      <c r="C62" s="10" t="str">
+        <f>_xll.qlBondPrice(C56,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R62C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B63" s="10">
+        <f>_xll.qlBondYield2(B37,B62,"actual360","CONTINUOUS","annual")</f>
+        <v>0.28928264826921379</v>
+      </c>
+      <c r="C63" s="10">
+        <f>_xll.qlBondYield2(C37,C62,"actual360","CONTINUOUS","annual")</f>
+        <v>0.28930497525756377</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B64" s="2">
+        <v>45667</v>
+      </c>
+      <c r="C64" s="2">
+        <v>45667</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B65" s="10">
+        <f>_xll.qlBondAccruedAmount(B37,B64)</f>
+        <v>0</v>
+      </c>
+      <c r="C65" s="10">
+        <f>_xll.qlBondAccruedAmount(C37,C64)</f>
+        <v>1.6666666666775853E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B66" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(B37)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C66" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C37)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B67" s="10">
+        <f>_xll.qlBondSettlementValue2(B37,B56)</f>
+        <v>77.244512464178655</v>
+      </c>
+      <c r="C67" s="10">
+        <f>_xll.qlBondSettlementValue2(C37,C56)</f>
+        <v>77.503599021422431</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A5:A7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F09BC366-53EA-43EA-8BCB-0489C1B271E0}">
+  <dimension ref="A3:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="45.42578125" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" t="str">
+        <f>_xll.qlBondPrice(100,"clean")</f>
+        <v>欣[test_bonds.xlsx]Callability!R3C2BondPrice,A</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" s="9">
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" t="str">
+        <f>_xll.qlCallability(B3,B4,B5)</f>
+        <v>欣[test_bonds.xlsx]Callability!R6C2Callability,A</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" t="str">
+        <f>_xll.qlCallabilityPrice(B6)</f>
+        <v>欣[test_bonds.xlsx]Callability!R7C2BondPrice,A</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="9">
+        <f>_xll.qlCallabilityDate(B6)</f>
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" t="str">
+        <f>_xll.qlCallabilityType(B6)</f>
+        <v>PUT</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0A1FE9-B1FE-4762-AEA9-E4B3F6C519F7}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1086,7 +2094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4EF9C2-FD4D-4E7F-8154-C8E782972C6B}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1095,7 +2103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCE8D14D-DD7E-4024-86F3-1C5FBF784E5F}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1105,8 +2113,75 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44B77307-DD7A-406E-AD93-A17357F921C0}">
+  <dimension ref="A3:B8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="46" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="3" t="str">
+        <f>_xll.qlBondPrice(B3,B4)</f>
+        <v>欣[test_bonds.xlsx]BondPrice!R5C2BondPrice,A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="3">
+        <f>_xll.qlBondPriceAmount(B5)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="3" t="str">
+        <f>_xll.qlBondPriceType(B5)</f>
+        <v>CLEAN</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="3" t="b">
+        <f>_xll.qlBondPriceIsValid(B5)</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8683113-FD1C-4D88-8D42-F7763B404E4F}">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1615,9 +2690,18 @@
       <c r="A47" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="10">
+      <c r="B47" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(B25)</f>
-        <v>2.3346336353520432</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C47" s="10">
         <f>_xll.qlBondDirtyPrice(C25)</f>
@@ -1651,64 +2735,86 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" s="10" t="str">
+        <f>_xll.qlBondPrice(B44,"clean")</f>
+        <v>欣[test_bonds.xlsx]Bond!R50C2BondPrice,A</v>
+      </c>
+      <c r="C50" s="10" t="str">
+        <f>_xll.qlBondPrice(C44,"clean")</f>
+        <v>欣[test_bonds.xlsx]Bond!R50C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B50" s="10">
-        <f>_xll.qlBondYield2(B25,B47,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426559332721</v>
-      </c>
-      <c r="C50" s="10">
-        <f>_xll.qlBondYield2(C25,C47,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426559332721</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="11" t="s">
+      <c r="B51" s="10">
+        <f>_xll.qlBondYield2(B25,B50,"actual360","CONTINUOUS","annual")</f>
+        <v>0.26946953931176648</v>
+      </c>
+      <c r="C51" s="10">
+        <f>_xll.qlBondYield2(C25,C50,"actual360","CONTINUOUS","annual")</f>
+        <v>0.26946953931176648</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B52" s="2">
         <v>45667</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C52" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B52" s="10">
-        <f>_xll.qlBondAccruedAmount(B25,B51)</f>
-        <v>1.6666666666664831E-2</v>
-      </c>
-      <c r="C52" s="10">
-        <f>_xll.qlBondAccruedAmount(C25,C51)</f>
-        <v>1.6666666666664831E-2</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B53" s="10">
+        <f>_xll.qlBondAccruedAmount(B25,B52)</f>
+        <v>1.6666666666664831E-2</v>
+      </c>
+      <c r="C53" s="10">
+        <f>_xll.qlBondAccruedAmount(C25,C52)</f>
+        <v>1.6666666666664831E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B53" s="10">
+      <c r="B54" s="10" t="str">
         <f>_xll.qlBondSettlementValue(B25)</f>
-        <v>2.3346336353520432</v>
-      </c>
-      <c r="C53" s="10">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C54" s="10">
         <f>_xll.qlBondSettlementValue(C25)</f>
         <v>2.3346336353520432</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B54" s="10">
+      <c r="B55" s="10">
         <f>_xll.qlBondSettlementValue2(B25,B44)</f>
         <v>2.3346336353520432</v>
       </c>
-      <c r="C54" s="10">
+      <c r="C55" s="10">
         <f>_xll.qlBondSettlementValue2(C25,C44)</f>
         <v>2.3346336353520432</v>
       </c>
@@ -1719,13 +2825,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA0BDDB4-6035-4089-86B1-6246F3228CBC}">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.85546875" customWidth="1"/>
-    <col min="2" max="2" width="60" style="3" customWidth="1"/>
+    <col min="2" max="2" width="88.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="59.28515625" style="3" customWidth="1"/>
     <col min="4" max="7" width="11.42578125" style="3"/>
   </cols>
@@ -1838,7 +2944,7 @@
         <f>_xll.qlBondNextCouponRate(B11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: no coupon paid at cashflow date January 8th, 2026
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 203, in qlBondNextCouponRate
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 209, in qlBondNextCouponRate
     return bond.nextCouponRate(date)
            ~~~~~~~~~~~~~~~~~~~^^^^^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25841, in nextCouponRate
@@ -1851,7 +2957,7 @@
         <f>_xll.qlBondNextCouponRate(C11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: no coupon paid at cashflow date January 8th, 2026
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 203, in qlBondNextCouponRate
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 209, in qlBondNextCouponRate
     return bond.nextCouponRate(date)
            ~~~~~~~~~~~~~~~~~~~^^^^^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25841, in nextCouponRate
@@ -2127,9 +3233,18 @@
         <f>_xll.qlBondDirtyPrice(B11)</f>
         <v>76.755078422532549</v>
       </c>
-      <c r="C33" s="10">
+      <c r="C33" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(C11)</f>
-        <v>92.106094107039056</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -2149,74 +3264,128 @@
       <c r="A35" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="10">
+      <c r="B35" s="10" t="str">
         <f>_xll.qlBondYield(B11,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C35" s="10" t="str">
+        <f>_xll.qlBondYield(C11,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B36" s="10" t="str">
+        <f>_xll.qlBondPrice(B30,"clean")</f>
+        <v>欣[test_bonds.xlsx]ZeroCouponBond!R36C2BondPrice,A</v>
+      </c>
+      <c r="C36" s="10" t="str">
+        <f>_xll.qlBondPrice(C30,"clean")</f>
+        <v>欣[test_bonds.xlsx]ZeroCouponBond!R36C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="10">
+        <f>_xll.qlBondYield2(B11,B36,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
-      <c r="C35" s="10">
-        <f>_xll.qlBondYield(C11,"actual360","CONTINUOUS","annual")</f>
+      <c r="C37" s="10">
+        <f>_xll.qlBondYield2(C11,C36,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="10">
-        <f>_xll.qlBondYield2(B11,B33,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-      <c r="C36" s="10">
-        <f>_xll.qlBondYield2(C11,C33,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B38" s="2">
         <v>45667</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C38" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38" s="10">
-        <f>_xll.qlBondAccruedAmount(B11,B37)</f>
-        <v>0</v>
-      </c>
-      <c r="C38" s="10">
-        <f>_xll.qlBondAccruedAmount(C11,C37)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="10">
+        <f>_xll.qlBondAccruedAmount(B11,B38)</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="10">
+        <f>_xll.qlBondAccruedAmount(C11,C38)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="10">
+      <c r="B40" s="10" t="str">
         <f>_xll.qlBondSettlementValue(B11)</f>
-        <v>76.755078422532549</v>
-      </c>
-      <c r="C39" s="10">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C40" s="10">
         <f>_xll.qlBondSettlementValue(C11)</f>
         <v>92.106094107039056</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B40" s="10">
+      <c r="B41" s="10">
         <f>_xll.qlBondSettlementValue2(B11,B30)</f>
         <v>76.755078422532549</v>
       </c>
-      <c r="C40" s="10">
+      <c r="C41" s="10">
         <f>_xll.qlBondSettlementValue2(C11,C30)</f>
         <v>92.106094107039056</v>
       </c>
@@ -2226,9 +3395,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00EB77E5-949B-439C-BFA2-575F2A710E3C}">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43" customWidth="1"/>
@@ -2379,7 +3548,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="34" t="s">
         <v>67</v>
       </c>
       <c r="B15" s="3">
@@ -2390,7 +3559,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="28"/>
+      <c r="A16" s="34"/>
       <c r="B16" s="3">
         <v>0.5</v>
       </c>
@@ -2399,7 +3568,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="28"/>
+      <c r="A17" s="34"/>
       <c r="B17" s="3">
         <v>0.6</v>
       </c>
@@ -2776,9 +3945,18 @@
         <f>_xll.qlBondDirtyPrice(B27)</f>
         <v>121.40429393805222</v>
       </c>
-      <c r="C49" s="10">
+      <c r="C49" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(C27)</f>
-        <v>127.36781301760961</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2798,61 +3976,106 @@
       <c r="A51" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="10" t="str">
         <f>_xll.qlBondYield(B27,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C51" s="10" t="str">
+        <f>_xll.qlBondYield(C27,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B52" s="10" t="str">
+        <f>_xll.qlBondPrice(B46,"clean")</f>
+        <v>欣[test_bonds.xlsx]FixedRateBond!R52C2BondPrice,A</v>
+      </c>
+      <c r="C52" s="10" t="str">
+        <f>_xll.qlBondPrice(C46,"clean")</f>
+        <v>欣[test_bonds.xlsx]FixedRateBond!R52C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" s="10">
+        <f>_xll.qlBondYield2(B27,B52,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
-      <c r="C51" s="10">
-        <f>_xll.qlBondYield(C27,"actual360","CONTINUOUS","annual")</f>
+      <c r="C53" s="10">
+        <f>_xll.qlBondYield2(C27,C52,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" s="10">
-        <f>_xll.qlBondYield2(B27,B49,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-      <c r="C52" s="10">
-        <f>_xll.qlBondYield2(C27,C49,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="11" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B54" s="2">
         <v>45667</v>
       </c>
-      <c r="C53" s="2">
+      <c r="C54" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B54" s="10">
-        <f>_xll.qlBondAccruedAmount(B27,B53)</f>
-        <v>0.22222222222221255</v>
-      </c>
-      <c r="C54" s="10">
-        <f>_xll.qlBondAccruedAmount(C27,C53)</f>
-        <v>-9.777777777777775</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B55" s="10">
+        <f>_xll.qlBondAccruedAmount(B27,B54)</f>
+        <v>0.22222222222221255</v>
+      </c>
+      <c r="C55" s="10">
+        <f>_xll.qlBondAccruedAmount(C27,C54)</f>
+        <v>-9.777777777777775</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B55" s="10" t="str">
+      <c r="B56" s="10" t="str">
         <f>_xll.qlBondSettlementValue(B27)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 529, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -2861,20 +4084,29 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C55" s="10">
+      <c r="C56" s="10" t="str">
         <f>_xll.qlBondSettlementValue(C27)</f>
-        <v>127.36781301760961</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="10">
+      <c r="B57" s="10">
         <f>_xll.qlBondSettlementValue2(B27,B46)</f>
         <v>121.40429393805221</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C57" s="10">
         <f>_xll.qlBondSettlementValue2(C27,C46)</f>
         <v>127.36781301760959</v>
       </c>
@@ -2887,9 +4119,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{303A5445-988F-4FD7-9234-8C10A40DEB2F}">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" customWidth="1"/>
@@ -2926,7 +4158,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>84</v>
       </c>
       <c r="B5" s="3">
@@ -2937,7 +4169,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="3">
         <v>125</v>
       </c>
@@ -2946,7 +4178,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="3">
         <v>100</v>
       </c>
@@ -3058,7 +4290,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="34" t="s">
         <v>67</v>
       </c>
       <c r="B17" s="3">
@@ -3069,7 +4301,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
+      <c r="A18" s="34"/>
       <c r="B18" s="3">
         <v>0.5</v>
       </c>
@@ -3078,7 +4310,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="28"/>
+      <c r="A19" s="34"/>
       <c r="B19" s="3">
         <v>0.6</v>
       </c>
@@ -3147,7 +4379,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="34" t="s">
         <v>89</v>
       </c>
       <c r="C27" s="3">
@@ -3155,13 +4387,13 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="28"/>
+      <c r="A28" s="34"/>
       <c r="C28" s="3">
         <v>110</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="28"/>
+      <c r="A29" s="34"/>
       <c r="C29" s="3">
         <v>110</v>
       </c>
@@ -3330,7 +4562,7 @@
         <f>_xll.qlBondRedemption(B30)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -3343,7 +4575,7 @@
         <f>_xll.qlBondRedemption(C30)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -3476,9 +4708,18 @@
         <f>_xll.qlBondDirtyPrice(B30)</f>
         <v>116.28899295466947</v>
       </c>
-      <c r="C52" s="10">
+      <c r="C52" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(C30)</f>
-        <v>115.0531622834792</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -3502,70 +4743,117 @@
         <f>_xll.qlBondYield(B30,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
-      <c r="C54" s="10">
+      <c r="C54" s="10" t="str">
         <f>_xll.qlBondYield(C30,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
+      <c r="A55" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B55" s="10" t="str">
+        <f>_xll.qlBondPrice(B49,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingFixedRateBond!R55C2BondPrice,A</v>
+      </c>
+      <c r="C55" s="10" t="str">
+        <f>_xll.qlBondPrice(C49,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingFixedRateBond!R55C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B55" s="10">
-        <f>_xll.qlBondYield2(B30,B52,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-      <c r="C55" s="10">
-        <f>_xll.qlBondYield2(C30,C52,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="11" t="s">
+      <c r="B56" s="10">
+        <f>_xll.qlBondYield2(B30,B55,"actual360","CONTINUOUS","annual")</f>
+        <v>0.2650188827598095</v>
+      </c>
+      <c r="C56" s="10">
+        <f>_xll.qlBondYield2(C30,C55,"actual360","CONTINUOUS","annual")</f>
+        <v>0.1561166555979252</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B57" s="2">
         <v>45667</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C57" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B57" s="10">
-        <f>_xll.qlBondAccruedAmount(B30,B56)</f>
-        <v>0.22222222222221252</v>
-      </c>
-      <c r="C57" s="10">
-        <f>_xll.qlBondAccruedAmount(C30,C56)</f>
-        <v>-9.7777777777777732</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B58" s="10">
-        <f>_xll.qlBondSettlementValue(B30)</f>
-        <v>174.43348943200422</v>
+        <f>_xll.qlBondAccruedAmount(B30,B57)</f>
+        <v>0.22222222222221252</v>
       </c>
       <c r="C58" s="10">
-        <f>_xll.qlBondSettlementValue(C30)</f>
-        <v>172.57974342521879</v>
+        <f>_xll.qlBondAccruedAmount(C30,C57)</f>
+        <v>-9.7777777777777732</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B59" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(B30)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C59" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C30)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B59" s="10">
+      <c r="B60" s="10">
         <f>_xll.qlBondSettlementValue2(B30,B49)</f>
         <v>174.43348943200419</v>
       </c>
-      <c r="C59" s="10">
+      <c r="C60" s="10">
         <f>_xll.qlBondSettlementValue2(C30,C49)</f>
         <v>172.57974342521879</v>
       </c>
@@ -3580,9 +4868,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F76F30CA-2F79-453E-B116-2A48310E361D}">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.42578125" customWidth="1"/>
@@ -3619,7 +4907,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="34" t="s">
         <v>90</v>
       </c>
       <c r="B5" s="3">
@@ -3630,7 +4918,7 @@
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="3">
         <v>125</v>
       </c>
@@ -3639,7 +4927,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
+      <c r="A7" s="34"/>
       <c r="B7" s="3">
         <v>100</v>
       </c>
@@ -4059,7 +5347,7 @@
         <f>_xll.qlBondRedemption(B34)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -4072,7 +5360,7 @@
         <f>_xll.qlBondRedemption(C34)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -4231,70 +5519,108 @@
         <f>_xll.qlBondYield(B34,"actual360","CONTINUOUS","annual")</f>
         <v>0.28928264971926221</v>
       </c>
-      <c r="C58" s="10">
+      <c r="C58" s="10" t="str">
         <f>_xll.qlBondYield(C34,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="10" t="str">
+        <f>_xll.qlBondPrice(B53,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingFloatingRateBond!R59C2BondPrice,A</v>
+      </c>
+      <c r="C59" s="10" t="str">
+        <f>_xll.qlBondPrice(C53,"clean")</f>
+        <v>欣[test_bonds.xlsx]AmortizingFloatingRateBond!R59C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B59" s="10">
-        <f>_xll.qlBondYield2(B34,B56,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C59" s="10">
-        <f>_xll.qlBondYield2(C34,C56,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="11" t="s">
+      <c r="B60" s="10">
+        <f>_xll.qlBondYield2(B34,B59,"actual360","CONTINUOUS","annual")</f>
+        <v>0.29158154279763698</v>
+      </c>
+      <c r="C60" s="10">
+        <f>_xll.qlBondYield2(C34,C59,"actual360","CONTINUOUS","annual")</f>
+        <v>0.19027274083304402</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B61" s="2">
         <v>45667</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C61" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B61" s="10">
-        <f>_xll.qlBondAccruedAmount(B34,B60)</f>
-        <v>0.16666666666666657</v>
-      </c>
-      <c r="C61" s="10">
-        <f>_xll.qlBondAccruedAmount(C34,C60)</f>
-        <v>-7.3333333333333286</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B62" s="10">
+        <f>_xll.qlBondAccruedAmount(B34,B61)</f>
+        <v>0.16666666666666657</v>
+      </c>
+      <c r="C62" s="10">
+        <f>_xll.qlBondAccruedAmount(C34,C61)</f>
+        <v>-7.3333333333333286</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B63" s="10" t="str">
         <f>_xll.qlBondSettlementValue(B34)</f>
-        <v>150.24592768168819</v>
-      </c>
-      <c r="C62" s="10">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C63" s="10">
         <f>_xll.qlBondSettlementValue(C34)</f>
         <v>139.76397912193815</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="8" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B63" s="10">
+      <c r="B64" s="10">
         <f>_xll.qlBondSettlementValue2(B34,B53)</f>
         <v>150.24592768168822</v>
       </c>
-      <c r="C63" s="10">
+      <c r="C64" s="10">
         <f>_xll.qlBondSettlementValue2(C34,C53)</f>
         <v>139.76397912193815</v>
       </c>
@@ -4308,9 +5634,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05025377-E5EA-48F0-BE68-1C47A2C5C8E6}">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.28515625" customWidth="1"/>
@@ -4851,9 +6177,18 @@
         <f>_xll.qlBondCleanPrice(B31)</f>
         <v>99.998840118437755</v>
       </c>
-      <c r="C50" s="10">
+      <c r="C50" s="10" t="str">
         <f>_xll.qlBondCleanPrice(C31)</f>
-        <v>100.51087441193772</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -4884,9 +6219,18 @@
       <c r="A53" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B53" s="10">
+      <c r="B53" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(B31)</f>
-        <v>100.16550678510443</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C53" s="10">
         <f>_xll.qlBondDirtyPrice(C31)</f>
@@ -4914,72 +6258,171 @@
         <f>_xll.qlBondYield(B31,"actual360","CONTINUOUS","annual")</f>
         <v>0.28928264971926221</v>
       </c>
-      <c r="C55" s="10">
+      <c r="C55" s="10" t="str">
         <f>_xll.qlBondYield(C31,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
+      <c r="A56" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="10" t="str">
+        <f>_xll.qlBondPrice(B50,"clean")</f>
+        <v>欣[test_bonds.xlsx]FloatingRateBond!R56C2BondPrice,A</v>
+      </c>
+      <c r="C56" s="10" t="str">
+        <f>_xll.qlBondPrice(C50,"clean")</f>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B56" s="10">
-        <f>_xll.qlBondYield2(B31,B53,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C56" s="10">
-        <f>_xll.qlBondYield2(C31,C53,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="11" t="s">
+      <c r="B57" s="10">
+        <f>_xll.qlBondYield2(B31,B56,"actual360","CONTINUOUS","annual")</f>
+        <v>0.29112129323880687</v>
+      </c>
+      <c r="C57" s="10" t="str">
+        <f>_xll.qlBondYield2(C31,C56,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">TypeError: TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
+  Possible C/C++ prototypes are:
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 505, in qlBondYield2
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        price,
+        ^^^^^^
+    ...&lt;6 lines&gt;...
+        guess
+        ^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
+  Possible C/C++ prototypes are:
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
+</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B58" s="2">
         <v>45667</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C58" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B58" s="10">
-        <f>_xll.qlBondAccruedAmount(B31,B57)</f>
-        <v>0.16666666666666657</v>
-      </c>
-      <c r="C58" s="10">
-        <f>_xll.qlBondAccruedAmount(C31,C57)</f>
-        <v>-7.3333333333333277</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B59" s="10">
-        <f>_xll.qlBondSettlementValue(B31)</f>
-        <v>100.16550678510443</v>
+        <f>_xll.qlBondAccruedAmount(B31,B58)</f>
+        <v>0.16666666666666657</v>
       </c>
       <c r="C59" s="10">
-        <f>_xll.qlBondSettlementValue(C31)</f>
-        <v>93.177541078604392</v>
+        <f>_xll.qlBondAccruedAmount(C31,C58)</f>
+        <v>-7.3333333333333277</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B60" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(B31)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C60" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C31)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B61" s="10">
         <f>_xll.qlBondSettlementValue2(B31,B50)</f>
         <v>100.16550678510443</v>
       </c>
-      <c r="C60" s="10">
+      <c r="C61" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(C31,C50)</f>
-        <v>93.177541078604392</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
   </sheetData>
@@ -4987,9 +6430,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27515A30-3B44-433D-8DBF-ACC4ED7765FD}">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46.140625" customWidth="1"/>
@@ -5624,9 +7067,18 @@
         <f>_xll.qlBondCleanPrice(B36)</f>
         <v>158.97331982635237</v>
       </c>
-      <c r="C55" s="10">
+      <c r="C55" s="10" t="str">
         <f>_xll.qlBondCleanPrice(C36)</f>
-        <v>89.639709460333037</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -5657,13 +7109,31 @@
       <c r="A58" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B58" s="10">
+      <c r="B58" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(B36)</f>
-        <v>159.52887538190791</v>
-      </c>
-      <c r="C58" s="10">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C58" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(C36)</f>
-        <v>89.639709460333037</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -5693,867 +7163,153 @@
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B61" s="10" t="str">
+        <f>_xll.qlBondPrice(B55,"clean")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R61C2BondPrice,A</v>
+      </c>
+      <c r="C61" s="10" t="str">
+        <f>_xll.qlBondPrice(C55,"clean")</f>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="10">
-        <f>_xll.qlBondYield2(B36,B58,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C61" s="10">
-        <f>_xll.qlBondYield2(C36,C58,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928265005463161</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="11" t="s">
+      <c r="B62" s="10">
+        <f>_xll.qlBondYield2(B36,B61,"actual360","CONTINUOUS","annual")</f>
+        <v>0.29367879784610279</v>
+      </c>
+      <c r="C62" s="10" t="str">
+        <f>_xll.qlBondYield2(C36,C61,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">TypeError: TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
+  Possible C/C++ prototypes are:
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 505, in qlBondYield2
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        price,
+        ^^^^^^
+    ...&lt;6 lines&gt;...
+        guess
+        ^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
+  Possible C/C++ prototypes are:
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
+    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
+    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
+</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B63" s="2">
         <v>45667</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C63" s="2">
         <v>45667</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B63" s="10">
-        <f>_xll.qlBondAccruedAmount(B36,B62)</f>
-        <v>0.55555555555555358</v>
-      </c>
-      <c r="C63" s="10">
-        <f>_xll.qlBondAccruedAmount(C36,C62)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B64" s="10">
-        <f>_xll.qlBondSettlementValue(B36)</f>
-        <v>159.52887538190791</v>
+        <f>_xll.qlBondAccruedAmount(B36,B63)</f>
+        <v>0.55555555555555358</v>
       </c>
       <c r="C64" s="10">
-        <f>_xll.qlBondSettlementValue(C36)</f>
-        <v>89.639709460333037</v>
+        <f>_xll.qlBondAccruedAmount(C36,C63)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B65" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(B36)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C65" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C36)</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+    return bond.settlementValue()
+           ~~~~~~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
+    return _QuantLib.Bond_settlementValue(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B65" s="10">
+      <c r="B66" s="10">
         <f>_xll.qlBondSettlementValue2(B36,B55)</f>
         <v>159.52887538190791</v>
       </c>
-      <c r="C65" s="10">
+      <c r="C66" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(C36,C55)</f>
-        <v>89.639709460333037</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28ABD84F-1436-4AE1-BC17-091C65B56114}">
-  <dimension ref="A1:C66"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="48.5703125" customWidth="1"/>
-    <col min="2" max="2" width="69.140625" customWidth="1"/>
-    <col min="3" max="3" width="71.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="2">
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="2">
-        <f>_xll.qlSettingsSetEvaluationDate(B1)</f>
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="3">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B5" s="3">
-        <v>103</v>
-      </c>
-      <c r="C5" s="3">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
-      <c r="B6" s="3">
-        <v>102</v>
-      </c>
-      <c r="C6" s="3">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="3">
-        <v>101</v>
-      </c>
-      <c r="C7" s="3">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="12">
-        <v>45665</v>
-      </c>
-      <c r="C8" s="12">
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" s="12">
-        <v>46030</v>
-      </c>
-      <c r="C9" s="12">
-        <v>46030</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C11" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="6">
-        <v>0</v>
-      </c>
-      <c r="C15" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="3" t="str">
-        <f>_xll.qlSchedule(B8,B9,B10,B11,B12,B13,B14,B15)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R16C2Schedule,A</v>
-      </c>
-      <c r="C16" s="3" t="str">
-        <f>_xll.qlSchedule(C8,C9,C10,C11,C12,C13,C14,C15)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R16C3Schedule,A</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="6">
-        <v>2</v>
-      </c>
-      <c r="C19" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B21" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C21" s="6" t="str">
-        <f>_xll.qlCalendar("TARGET")</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="6" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R25C2Euribor,A</v>
-      </c>
-      <c r="C25" s="6" t="str">
-        <f>_xll.qlEuribor("3M")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R25C3Euribor,A</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B26" s="6" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Actual360","Compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R26C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C26" s="6" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.03,"Actual360","Compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R26C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>102</v>
-      </c>
-      <c r="B27" s="3" t="str">
-        <f>_xll.qlSwapIndex(B17,B18,B19,B20,B21,B22,B23,B24,B25,B26)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R27C2SwapIndex,A</v>
-      </c>
-      <c r="C27" s="3" t="str">
-        <f>_xll.qlSwapIndex(C17,C18,C19,C20,C21,C22,C23,C24,C25,C26)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R27C3SwapIndex,A</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>86</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>92</v>
-      </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>94</v>
-      </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3">
-        <v>3.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>97</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>17</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="2">
-        <v>45663</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B37" t="str">
-        <f>_xll.qlAmortizingCmsRateBond(B4,B5:B7,B16,B27,B28)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R37C2AmortizingCmsRateBond,A</v>
-      </c>
-      <c r="C37" t="str">
-        <f>_xll.qlAmortizingCmsRateBond(C4,C5:C7,C16,C27,C28,C29,C30,C31,C32,C33,C34,C35,C36)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R37C3AmortizingCmsRateBond,A</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="3">
-        <f>_xll.qlBondNextCouponRate(B37)</f>
-        <v>0</v>
-      </c>
-      <c r="C38" s="3">
-        <f>_xll.qlBondNextCouponRate(C37)</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B39" s="3">
-        <f>_xll.qlBondPreviousCouponRate(B37)</f>
-        <v>0</v>
-      </c>
-      <c r="C39" s="3">
-        <f>_xll.qlBondPreviousCouponRate(C37)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" s="2">
-        <f>_xll.qlBondNextCashFlowDate(B37)</f>
-        <v>45755</v>
-      </c>
-      <c r="C40" s="2">
-        <f>_xll.qlBondNextCashFlowDate(C37)</f>
-        <v>45755</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B41" s="2">
-        <f>_xll.qlBondPreviousCashFlowDate(B37)</f>
-        <v>0</v>
-      </c>
-      <c r="C41" s="2">
-        <f>_xll.qlBondPreviousCashFlowDate(C37)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B42" s="3">
-        <f>_xll.qlBondSettlementDays(B37)</f>
-        <v>2</v>
-      </c>
-      <c r="C42" s="3">
-        <f>_xll.qlBondSettlementDays(C37)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B43" s="2">
-        <f>_xll.qlBondSettlementDate(B37)</f>
-        <v>45667</v>
-      </c>
-      <c r="C43" s="2">
-        <f>_xll.qlBondSettlementDate(C37)</f>
-        <v>45667</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B44" s="3" t="b">
-        <f>_xll.qlBondIsTradable(B37)</f>
-        <v>1</v>
-      </c>
-      <c r="C44" s="3" t="b">
-        <f>_xll.qlBondIsTradable(C37)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B45" s="2">
-        <f>_xll.qlBondStartDate(B37)</f>
-        <v>45665</v>
-      </c>
-      <c r="C45" s="2">
-        <f>_xll.qlBondStartDate(C37)</f>
-        <v>45665</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B46" s="2">
-        <f>_xll.qlBondMaturityDate(B37)</f>
-        <v>46030</v>
-      </c>
-      <c r="C46" s="2">
-        <f>_xll.qlBondMaturityDate(C37)</f>
-        <v>46030</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B47" s="3">
-        <f>_xll.qlBondIssueDate(B37)</f>
-        <v>0</v>
-      </c>
-      <c r="C47" s="3">
-        <f>_xll.qlBondIssueDate(C37)</f>
-        <v>45663</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B48" s="3" t="str">
-        <f>_xll.qlBondCashFlows(B37)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R48C2CashFlow,A</v>
-      </c>
-      <c r="C48" s="3" t="str">
-        <f>_xll.qlBondCashFlows(C37)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R48C3CashFlow,A</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="3" t="str">
-        <f>_xll.qlBondRedemption(B37)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
-    return bond.redemption()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
-    return _QuantLib.Bond_redemption(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: multiple redemption cash flows given
-</v>
-      </c>
-      <c r="C49" s="3" t="str">
-        <f>_xll.qlBondRedemption(C37)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 320, in qlBondRedemption
-    return bond.redemption()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
-    return _QuantLib.Bond_redemption(self)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^
-RuntimeError: multiple redemption cash flows given
-</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B50" s="3" t="str">
-        <f>_xll.qlBondRedemptions(B37)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R50C2CashFlow,A</v>
-      </c>
-      <c r="C50" s="3" t="str">
-        <f>_xll.qlBondRedemptions(C37)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R50C3CashFlow,A</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B51" s="3" t="str">
-        <f>_xll.qlBondCalendar(B37)</f>
-        <v>TARGET</v>
-      </c>
-      <c r="C51" s="3" t="str">
-        <f>_xll.qlBondCalendar(C37)</f>
-        <v>TARGET</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B52" s="3">
-        <f>_xll.qlBondNotional(B37)</f>
-        <v>103</v>
-      </c>
-      <c r="C52" s="3">
-        <f>_xll.qlBondNotional(C37)</f>
-        <v>103</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B53" s="3">
-        <f>_xll.qlBondNotionals(B37)</f>
-        <v>103</v>
-      </c>
-      <c r="C53" s="3">
-        <f>_xll.qlBondNotionals(C37)</f>
-        <v>103</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B54" s="3" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.3,"actual360","compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R54C2YieldTermStructureHandle,A</v>
-      </c>
-      <c r="C54" s="3" t="str">
-        <f>_xll.qlFlatForward(#REF!,0.3,"actual360","compounded","Quarterly")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R54C3YieldTermStructureHandle,A</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B55" s="3" t="str">
-        <f>_xll.qlBondSetDiscountingEngine(B37,B54)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R55C2DiscountingBondEngine,A</v>
-      </c>
-      <c r="C55" s="3" t="str">
-        <f>_xll.qlBondSetDiscountingEngine(C37,C54)</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R55C3DiscountingBondEngine,A</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B56" s="10">
-        <f>_xll.qlBondCleanPrice(B37)</f>
-        <v>74.994672295319077</v>
-      </c>
-      <c r="C56" s="10">
-        <f>_xll.qlBondCleanPrice(C37)</f>
-        <v>75.244545975491022</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B57" s="10">
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C57" s="10">
-        <v>0.28928264971926221</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B58" s="10">
-        <f>_xll.qlBondCleanPrice2(B37,B57,"actual360","continuous")</f>
-        <v>74.994672041966595</v>
-      </c>
-      <c r="C58" s="10">
-        <f>_xll.qlBondCleanPrice2(C37,C57,"actual360","continuous")</f>
-        <v>75.244545721623112</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B59" s="10">
-        <f>_xll.qlBondDirtyPrice(B37)</f>
-        <v>74.994672295319077</v>
-      </c>
-      <c r="C59" s="10">
-        <f>_xll.qlBondDirtyPrice(C37)</f>
-        <v>75.246212642157701</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B60" s="10">
-        <f>_xll.qlBondDirtyPrice2(B37,B57,"actual360","CONTINUOUS","annual")</f>
-        <v>74.994672041966595</v>
-      </c>
-      <c r="C60" s="10">
-        <f>_xll.qlBondDirtyPrice2(C37,C57,"actual360","CONTINUOUS","annual")</f>
-        <v>75.246212388289791</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B61" s="10">
-        <f>_xll.qlBondYield(B37,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264826921379</v>
-      </c>
-      <c r="C61" s="10">
-        <f>_xll.qlBondYield(C37,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264793774228</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B62" s="10">
-        <f>_xll.qlBondYield2(B37,B59,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264826921379</v>
-      </c>
-      <c r="C62" s="10">
-        <f>_xll.qlBondYield2(C37,C59,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264793774228</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B63" s="2">
-        <v>45667</v>
-      </c>
-      <c r="C63" s="2">
-        <v>45667</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B64" s="10">
-        <f>_xll.qlBondAccruedAmount(B37,B63)</f>
-        <v>0</v>
-      </c>
-      <c r="C64" s="10">
-        <f>_xll.qlBondAccruedAmount(C37,C63)</f>
-        <v>1.6666666666775853E-3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B65" s="10">
-        <f>_xll.qlBondSettlementValue(B37)</f>
-        <v>77.244512464178641</v>
-      </c>
-      <c r="C65" s="10">
-        <f>_xll.qlBondSettlementValue(C37)</f>
-        <v>77.503599021422431</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B66" s="10">
-        <f>_xll.qlBondSettlementValue2(B37,B56)</f>
-        <v>77.244512464178655</v>
-      </c>
-      <c r="C66" s="10">
-        <f>_xll.qlBondSettlementValue2(C37,C56)</f>
-        <v>77.503599021422431</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A5:A7"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Modify functions arguments types and names for consistency reasons.
</commit_message>
<xml_diff>
--- a/tests/workbooks/test_bonds.xlsx
+++ b/tests/workbooks/test_bonds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{804525A8-9446-4835-9374-D51F9E284B26}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0FF61BC-DA5F-472D-B229-DD580FBE5AA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="32370" windowHeight="9360" xr2:uid="{A8952777-E146-413E-A9B0-D4A573A66C27}"/>
   </bookViews>
@@ -1685,7 +1685,7 @@
         <f>_xll.qlBondIssueDate(B37)</f>
         <v>0</v>
       </c>
-      <c r="C47" s="3">
+      <c r="C47" s="2">
         <f>_xll.qlBondIssueDate(C37)</f>
         <v>45663</v>
       </c>
@@ -1711,7 +1711,7 @@
         <f>_xll.qlBondRedemption(B37)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -1724,7 +1724,7 @@
         <f>_xll.qlBondRedemption(C37)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -1820,9 +1820,18 @@
         <f>_xll.qlBondCleanPrice(B37)</f>
         <v>74.994672295319077</v>
       </c>
-      <c r="C56" s="10">
+      <c r="C56" s="10" t="str">
         <f>_xll.qlBondCleanPrice(C37)</f>
-        <v>75.244545975491022</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1879,11 +1888,15 @@
       <c r="A61" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B61" s="10" t="str">
+      <c r="B61" s="10">
         <f>_xll.qlBondYield(B37,"actual360","CONTINUOUS","annual")</f>
+        <v>0.28928264826921379</v>
+      </c>
+      <c r="C61" s="10" t="str">
+        <f>_xll.qlBondYield(C37,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -1899,10 +1912,6 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C61" s="10">
-        <f>_xll.qlBondYield(C37,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264793774228</v>
-      </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
@@ -1914,7 +1923,16 @@
       </c>
       <c r="C62" s="10" t="str">
         <f>_xll.qlBondPrice(C56,"clean")</f>
-        <v>欣[test_bonds.xlsx]AmortizingCmsRateBond!R62C3BondPrice,A</v>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1925,9 +1943,18 @@
         <f>_xll.qlBondYield2(B37,B62,"actual360","CONTINUOUS","annual")</f>
         <v>0.28928264826921379</v>
       </c>
-      <c r="C63" s="10">
+      <c r="C63" s="10" t="str">
         <f>_xll.qlBondYield2(C37,C62,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28930497525756377</v>
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1958,11 +1985,15 @@
       <c r="A66" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B66" s="10" t="str">
+      <c r="B66" s="10">
         <f>_xll.qlBondSettlementValue(B37)</f>
+        <v>77.244512464178641</v>
+      </c>
+      <c r="C66" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C37)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -1971,19 +2002,6 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C66" s="10" t="str">
-        <f>_xll.qlBondSettlementValue(C37)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
-    return bond.settlementValue()
-           ~~~~~~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
-    return _QuantLib.Bond_settlementValue(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
@@ -1993,9 +2011,18 @@
         <f>_xll.qlBondSettlementValue2(B37,B56)</f>
         <v>77.244512464178655</v>
       </c>
-      <c r="C67" s="10">
+      <c r="C67" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(C37,C56)</f>
-        <v>77.503599021422431</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
   </sheetData>
@@ -2012,7 +2039,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="45.42578125" customWidth="1"/>
+    <col min="2" max="2" width="45.42578125" style="3" customWidth="1"/>
     <col min="6" max="6" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2020,7 +2047,7 @@
       <c r="A3" t="s">
         <v>127</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B3" s="3" t="str">
         <f>_xll.qlBondPrice(100,"clean")</f>
         <v>欣[test_bonds.xlsx]Callability!R3C2BondPrice,A</v>
       </c>
@@ -2029,7 +2056,7 @@
       <c r="A4" t="s">
         <v>128</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2037,7 +2064,7 @@
       <c r="A5" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="2">
         <v>46357</v>
       </c>
     </row>
@@ -2045,7 +2072,7 @@
       <c r="A6" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B6" s="3" t="str">
         <f>_xll.qlCallability(B3,B4,B5)</f>
         <v>欣[test_bonds.xlsx]Callability!R6C2Callability,A</v>
       </c>
@@ -2054,7 +2081,7 @@
       <c r="A7" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B7" s="3" t="str">
         <f>_xll.qlCallabilityPrice(B6)</f>
         <v>欣[test_bonds.xlsx]Callability!R7C2BondPrice,A</v>
       </c>
@@ -2063,7 +2090,7 @@
       <c r="A8" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="2">
         <f>_xll.qlCallabilityDate(B6)</f>
         <v>46357</v>
       </c>
@@ -2072,7 +2099,7 @@
       <c r="A9" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B9" s="3" t="str">
         <f>_xll.qlCallabilityType(B6)</f>
         <v>PUT</v>
       </c>
@@ -2653,9 +2680,18 @@
       <c r="A44" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="10">
+      <c r="B44" s="10" t="str">
         <f>_xll.qlBondCleanPrice(B25)</f>
-        <v>2.3179669686853783</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C44" s="10">
         <f>_xll.qlBondCleanPrice(C25)</f>
@@ -2690,18 +2726,9 @@
       <c r="A47" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B47" s="10" t="str">
+      <c r="B47" s="10">
         <f>_xll.qlBondDirtyPrice(B25)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
-    return bond.dirtyPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
-    return _QuantLib.Bond_dirtyPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>2.3346336353520432</v>
       </c>
       <c r="C47" s="10">
         <f>_xll.qlBondDirtyPrice(C25)</f>
@@ -2725,9 +2752,25 @@
       <c r="A49" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B49" s="10">
+      <c r="B49" s="10" t="str">
         <f>_xll.qlBondYield(B25,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426559332721</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C49" s="10">
         <f>_xll.qlBondYield(C25,"actual360","CONTINUOUS","annual")</f>
@@ -2740,7 +2783,16 @@
       </c>
       <c r="B50" s="10" t="str">
         <f>_xll.qlBondPrice(B44,"clean")</f>
-        <v>欣[test_bonds.xlsx]Bond!R50C2BondPrice,A</v>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
       <c r="C50" s="10" t="str">
         <f>_xll.qlBondPrice(C44,"clean")</f>
@@ -2751,9 +2803,18 @@
       <c r="A51" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="10">
+      <c r="B51" s="10" t="str">
         <f>_xll.qlBondYield2(B25,B50,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26946953931176648</v>
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
       </c>
       <c r="C51" s="10">
         <f>_xll.qlBondYield2(C25,C50,"actual360","CONTINUOUS","annual")</f>
@@ -2788,11 +2849,15 @@
       <c r="A54" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B54" s="10" t="str">
+      <c r="B54" s="10">
         <f>_xll.qlBondSettlementValue(B25)</f>
+        <v>2.3346336353520432</v>
+      </c>
+      <c r="C54" s="10" t="str">
+        <f>_xll.qlBondSettlementValue(C25)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -2801,18 +2866,23 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C54" s="10">
-        <f>_xll.qlBondSettlementValue(C25)</f>
-        <v>2.3346336353520432</v>
-      </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(B25,B44)</f>
-        <v>2.3346336353520432</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
       <c r="C55" s="10">
         <f>_xll.qlBondSettlementValue2(C25,C44)</f>
@@ -2944,7 +3014,7 @@
         <f>_xll.qlBondNextCouponRate(B11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: no coupon paid at cashflow date January 8th, 2026
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 209, in qlBondNextCouponRate
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 249, in qlBondNextCouponRate
     return bond.nextCouponRate(date)
            ~~~~~~~~~~~~~~~~~~~^^^^^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25841, in nextCouponRate
@@ -2957,7 +3027,7 @@
         <f>_xll.qlBondNextCouponRate(C11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: no coupon paid at cashflow date January 8th, 2026
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 209, in qlBondNextCouponRate
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 249, in qlBondNextCouponRate
     return bond.nextCouponRate(date)
            ~~~~~~~~~~~~~~~~~~~^^^^^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25841, in nextCouponRate
@@ -3196,9 +3266,18 @@
         <f>_xll.qlBondCleanPrice(B11)</f>
         <v>76.755078422532549</v>
       </c>
-      <c r="C30" s="10">
+      <c r="C30" s="10" t="str">
         <f>_xll.qlBondCleanPrice(C11)</f>
-        <v>92.106094107039056</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -3229,15 +3308,11 @@
       <c r="A33" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="10">
+      <c r="B33" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(B11)</f>
-        <v>76.755078422532549</v>
-      </c>
-      <c r="C33" s="10" t="str">
-        <f>_xll.qlBondDirtyPrice(C11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 511, in qlBondDirtyPrice
     return bond.dirtyPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
@@ -3246,6 +3321,10 @@
 RuntimeError: null pricing engine
 </v>
       </c>
+      <c r="C33" s="10">
+        <f>_xll.qlBondDirtyPrice(C11)</f>
+        <v>92.106094107039056</v>
+      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
@@ -3268,7 +3347,7 @@
         <f>_xll.qlBondYield(B11,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -3284,25 +3363,9 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C35" s="10" t="str">
+      <c r="C35" s="10">
         <f>_xll.qlBondYield(C11,"actual360","CONTINUOUS","annual")</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
-    return bond.bondYield(
-           ~~~~~~~~~~~~~~^
-        dc,
-        ^^^
-    ...&lt;3 lines&gt;...
-        max_evaluations
-        ^^^^^^^^^^^^^^^
-    )
-    ^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
-    return _QuantLib.Bond_bondYield(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>0.26236426417183883</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -3315,7 +3378,16 @@
       </c>
       <c r="C36" s="10" t="str">
         <f>_xll.qlBondPrice(C30,"clean")</f>
-        <v>欣[test_bonds.xlsx]ZeroCouponBond!R36C3BondPrice,A</v>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -3326,9 +3398,18 @@
         <f>_xll.qlBondYield2(B11,B36,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
-      <c r="C37" s="10">
+      <c r="C37" s="10" t="str">
         <f>_xll.qlBondYield2(C11,C36,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -3363,7 +3444,7 @@
         <f>_xll.qlBondSettlementValue(B11)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -3385,9 +3466,18 @@
         <f>_xll.qlBondSettlementValue2(B11,B30)</f>
         <v>76.755078422532549</v>
       </c>
-      <c r="C41" s="10">
+      <c r="C41" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(C11,C30)</f>
-        <v>92.106094107039056</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
   </sheetData>
@@ -3908,9 +3998,18 @@
         <f>_xll.qlBondCleanPrice(B27)</f>
         <v>121.40429393805222</v>
       </c>
-      <c r="C46" s="10">
+      <c r="C46" s="10" t="str">
         <f>_xll.qlBondCleanPrice(C27)</f>
-        <v>127.36781301760961</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -3945,18 +4044,9 @@
         <f>_xll.qlBondDirtyPrice(B27)</f>
         <v>121.40429393805222</v>
       </c>
-      <c r="C49" s="10" t="str">
+      <c r="C49" s="10">
         <f>_xll.qlBondDirtyPrice(C27)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
-    return bond.dirtyPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
-    return _QuantLib.Bond_dirtyPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>127.36781301760961</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -3976,11 +4066,15 @@
       <c r="A51" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="10" t="str">
+      <c r="B51" s="10">
         <f>_xll.qlBondYield(B27,"actual360","CONTINUOUS","annual")</f>
+        <v>0.26236426417183883</v>
+      </c>
+      <c r="C51" s="10" t="str">
+        <f>_xll.qlBondYield(C27,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -3996,26 +4090,6 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C51" s="10" t="str">
-        <f>_xll.qlBondYield(C27,"actual360","CONTINUOUS","annual")</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
-    return bond.bondYield(
-           ~~~~~~~~~~~~~~^
-        dc,
-        ^^^
-    ...&lt;3 lines&gt;...
-        max_evaluations
-        ^^^^^^^^^^^^^^^
-    )
-    ^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
-    return _QuantLib.Bond_bondYield(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
@@ -4027,7 +4101,16 @@
       </c>
       <c r="C52" s="10" t="str">
         <f>_xll.qlBondPrice(C46,"clean")</f>
-        <v>欣[test_bonds.xlsx]FixedRateBond!R52C3BondPrice,A</v>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -4038,9 +4121,18 @@
         <f>_xll.qlBondYield2(B27,B52,"actual360","CONTINUOUS","annual")</f>
         <v>0.26236426417183883</v>
       </c>
-      <c r="C53" s="10">
+      <c r="C53" s="10" t="str">
         <f>_xll.qlBondYield2(C27,C52,"actual360","CONTINUOUS","annual")</f>
-        <v>0.26236426417183883</v>
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -4071,31 +4163,13 @@
       <c r="A56" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B56" s="10" t="str">
+      <c r="B56" s="10">
         <f>_xll.qlBondSettlementValue(B27)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
-    return bond.settlementValue()
-           ~~~~~~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
-    return _QuantLib.Bond_settlementValue(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-      <c r="C56" s="10" t="str">
+        <v>121.40429393805221</v>
+      </c>
+      <c r="C56" s="10">
         <f>_xll.qlBondSettlementValue(C27)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
-    return bond.settlementValue()
-           ~~~~~~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
-    return _QuantLib.Bond_settlementValue(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>127.36781301760961</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -4106,9 +4180,18 @@
         <f>_xll.qlBondSettlementValue2(B27,B46)</f>
         <v>121.40429393805221</v>
       </c>
-      <c r="C57" s="10">
+      <c r="C57" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(C27,C46)</f>
-        <v>127.36781301760959</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
     </row>
   </sheetData>
@@ -4375,7 +4458,7 @@
         <v>73</v>
       </c>
       <c r="C26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -4562,7 +4645,7 @@
         <f>_xll.qlBondRedemption(B30)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -4575,7 +4658,7 @@
         <f>_xll.qlBondRedemption(C30)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -4708,18 +4791,9 @@
         <f>_xll.qlBondDirtyPrice(B30)</f>
         <v>116.28899295466947</v>
       </c>
-      <c r="C52" s="10" t="str">
+      <c r="C52" s="10">
         <f>_xll.qlBondDirtyPrice(C30)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
-    return bond.dirtyPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
-    return _QuantLib.Bond_dirtyPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>115.0531622834792</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -4747,7 +4821,7 @@
         <f>_xll.qlBondYield(C30,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -4818,31 +4892,13 @@
       <c r="A59" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B59" s="10" t="str">
+      <c r="B59" s="10">
         <f>_xll.qlBondSettlementValue(B30)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
-    return bond.settlementValue()
-           ~~~~~~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
-    return _QuantLib.Bond_settlementValue(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
-      </c>
-      <c r="C59" s="10" t="str">
+        <v>174.43348943200422</v>
+      </c>
+      <c r="C59" s="10">
         <f>_xll.qlBondSettlementValue(C30)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
-    return bond.settlementValue()
-           ~~~~~~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
-    return _QuantLib.Bond_settlementValue(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>172.57974342521879</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -5192,7 +5248,7 @@
         <v>欣[test_bonds.xlsx]AmortizingFloatingRateBond!R34C2AmortizingFloatingRateBond,A</v>
       </c>
       <c r="C34" s="3" t="str">
-        <f>_xll.qlAmortizingFloatingRateBond(C4,C5:C7,C16,C18,C19,C20,C21,C22,C23,,,C26,C27,C28,C29,C30,C31,C32,C33)</f>
+        <f>_xll.qlAmortizingFloatingRateBond(C4,C5:C7,C16,C18,C19,C20,C21,C22,C23,C24,C25,C26,C27,C28,C29,C30,C31,C32,C33)</f>
         <v>欣[test_bonds.xlsx]AmortizingFloatingRateBond!R34C3AmortizingFloatingRateBond,A</v>
       </c>
     </row>
@@ -5347,7 +5403,7 @@
         <f>_xll.qlBondRedemption(B34)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -5360,7 +5416,7 @@
         <f>_xll.qlBondRedemption(C34)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: multiple redemption cash flows given
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 326, in qlBondRedemption
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 402, in qlBondRedemption
     return bond.redemption()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25889, in redemption
@@ -5452,9 +5508,18 @@
       <c r="A53" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="10">
+      <c r="B53" s="10" t="str">
         <f>_xll.qlBondCleanPrice(B34)</f>
-        <v>99.997285121125458</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C53" s="10">
         <f>_xll.qlBondCleanPrice(C34)</f>
@@ -5489,9 +5554,18 @@
       <c r="A56" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B56" s="10">
+      <c r="B56" s="10" t="str">
         <f>_xll.qlBondDirtyPrice(B34)</f>
-        <v>100.16395178779213</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 511, in qlBondDirtyPrice
+    return bond.dirtyPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
+    return _QuantLib.Bond_dirtyPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
       <c r="C56" s="10">
         <f>_xll.qlBondDirtyPrice(C34)</f>
@@ -5515,15 +5589,11 @@
       <c r="A58" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B58" s="10">
+      <c r="B58" s="10" t="str">
         <f>_xll.qlBondYield(B34,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C58" s="10" t="str">
-        <f>_xll.qlBondYield(C34,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -5539,6 +5609,26 @@
 RuntimeError: null pricing engine
 </v>
       </c>
+      <c r="C58" s="10" t="str">
+        <f>_xll.qlBondYield(C34,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
@@ -5546,7 +5636,16 @@
       </c>
       <c r="B59" s="10" t="str">
         <f>_xll.qlBondPrice(B53,"clean")</f>
-        <v>欣[test_bonds.xlsx]AmortizingFloatingRateBond!R59C2BondPrice,A</v>
+        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
       <c r="C59" s="10" t="str">
         <f>_xll.qlBondPrice(C53,"clean")</f>
@@ -5557,9 +5656,18 @@
       <c r="A60" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="10" t="str">
         <f>_xll.qlBondYield2(B34,B59,"actual360","CONTINUOUS","annual")</f>
-        <v>0.29158154279763698</v>
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
       </c>
       <c r="C60" s="10">
         <f>_xll.qlBondYield2(C34,C59,"actual360","CONTINUOUS","annual")</f>
@@ -5598,7 +5706,7 @@
         <f>_xll.qlBondSettlementValue(B34)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -5616,9 +5724,18 @@
       <c r="A64" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B64" s="10">
+      <c r="B64" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(B34,B53)</f>
-        <v>150.24592768168822</v>
+        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float</v>
       </c>
       <c r="C64" s="10">
         <f>_xll.qlBondSettlementValue2(C34,C53)</f>
@@ -5931,7 +6048,7 @@
         <v>欣[test_bonds.xlsx]FloatingRateBond!R31C2FloatingRateBond,A</v>
       </c>
       <c r="C31" s="3" t="str">
-        <f>_xll.qlFloatingRateBond(C4,C5,C14,C16,C17,C18,C19,C20,C21,,,C24,C25,C26,C27,C28,C29,C30)</f>
+        <f>_xll.qlFloatingRateBond(C4,C5,C14,C16,C17,C18,C19,C20,C21,C22,C23,C24,C25,C26,C27,C28,C29,C30)</f>
         <v>欣[test_bonds.xlsx]FloatingRateBond!R31C3FloatingRateBond,A</v>
       </c>
     </row>
@@ -6177,18 +6294,9 @@
         <f>_xll.qlBondCleanPrice(B31)</f>
         <v>99.998840118437755</v>
       </c>
-      <c r="C50" s="10" t="str">
+      <c r="C50" s="10">
         <f>_xll.qlBondCleanPrice(C31)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
-    return bond.cleanPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
-    return _QuantLib.Bond_cleanPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>100.51087441193772</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -6223,7 +6331,7 @@
         <f>_xll.qlBondDirtyPrice(B31)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 511, in qlBondDirtyPrice
     return bond.dirtyPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
@@ -6254,15 +6362,11 @@
       <c r="A55" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="10" t="str">
         <f>_xll.qlBondYield(B31,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C55" s="10" t="str">
-        <f>_xll.qlBondYield(C31,"actual360","CONTINUOUS","annual")</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondYield
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
         dc,
@@ -6278,74 +6382,51 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="B56" s="10" t="str">
-        <f>_xll.qlBondPrice(B50,"clean")</f>
-        <v>欣[test_bonds.xlsx]FloatingRateBond!R56C2BondPrice,A</v>
-      </c>
-      <c r="C56" s="10" t="str">
-        <f>_xll.qlBondPrice(C50,"clean")</f>
-        <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+      <c r="C55" s="10" t="str">
+        <f>_xll.qlBondYield(C31,"actual360","CONTINUOUS","annual")</f>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
-    return bond.cleanPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
-    return _QuantLib.Bond_cleanPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-': Expected float</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" s="10">
-        <f>_xll.qlBondYield2(B31,B56,"actual360","CONTINUOUS","annual")</f>
-        <v>0.29112129323880687</v>
-      </c>
-      <c r="C57" s="10" t="str">
-        <f>_xll.qlBondYield2(C31,C56,"actual360","CONTINUOUS","annual")</f>
-        <v xml:space="preserve">TypeError: TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
-  Possible C/C++ prototypes are:
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 505, in qlBondYield2
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
     return bond.bondYield(
            ~~~~~~~~~~~~~~^
-        price,
-        ^^^^^^
-    ...&lt;6 lines&gt;...
-        guess
-        ^^^^^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
     )
     ^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
     return _QuantLib.Bond_bondYield(self, *args)
            ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
-  Possible C/C++ prototypes are:
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
+RuntimeError: null pricing engine
 </v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B56" s="10" t="str">
+        <f>_xll.qlBondPrice(B50,"clean")</f>
+        <v>欣[test_bonds.xlsx]FloatingRateBond!R56C2BondPrice,A</v>
+      </c>
+      <c r="C56" s="10" t="str">
+        <f>_xll.qlBondPrice(C50,"clean")</f>
+        <v>欣[test_bonds.xlsx]FloatingRateBond!R56C3BondPrice,A</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" s="10">
+        <f>_xll.qlBondYield2(B31,B56,"actual360","CONTINUOUS","annual")</f>
+        <v>0.29112129323880687</v>
+      </c>
+      <c r="C57" s="10">
+        <f>_xll.qlBondYield2(C31,C56,"actual360","CONTINUOUS","annual")</f>
+        <v>0.21004909842705732</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -6380,7 +6461,7 @@
         <f>_xll.qlBondSettlementValue(B31)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -6393,7 +6474,7 @@
         <f>_xll.qlBondSettlementValue(C31)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -6411,18 +6492,9 @@
         <f>_xll.qlBondSettlementValue2(B31,B50)</f>
         <v>100.16550678510443</v>
       </c>
-      <c r="C61" s="10" t="str">
+      <c r="C61" s="10">
         <f>_xll.qlBondSettlementValue2(C31,C50)</f>
-        <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
-    return bond.cleanPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
-    return _QuantLib.Bond_cleanPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-': Expected float</v>
+        <v>93.177541078604392</v>
       </c>
     </row>
   </sheetData>
@@ -7063,15 +7135,11 @@
       <c r="A55" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B55" s="10">
+      <c r="B55" s="10" t="str">
         <f>_xll.qlBondCleanPrice(B36)</f>
-        <v>158.97331982635237</v>
-      </c>
-      <c r="C55" s="10" t="str">
-        <f>_xll.qlBondCleanPrice(C36)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
     return bond.cleanPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
@@ -7080,6 +7148,10 @@
 RuntimeError: null pricing engine
 </v>
       </c>
+      <c r="C55" s="10">
+        <f>_xll.qlBondCleanPrice(C36)</f>
+        <v>89.639709460333037</v>
+      </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
@@ -7113,7 +7185,7 @@
         <f>_xll.qlBondDirtyPrice(B36)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 511, in qlBondDirtyPrice
     return bond.dirtyPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
@@ -7122,18 +7194,9 @@
 RuntimeError: null pricing engine
 </v>
       </c>
-      <c r="C58" s="10" t="str">
+      <c r="C58" s="10">
         <f>_xll.qlBondDirtyPrice(C36)</f>
-        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 418, in qlBondDirtyPrice
-    return bond.dirtyPrice()
-           ~~~~~~~~~~~~~~~^^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25915, in dirtyPrice
-    return _QuantLib.Bond_dirtyPrice(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-RuntimeError: null pricing engine
-</v>
+        <v>89.639709460333037</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -7153,13 +7216,45 @@
       <c r="A60" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B60" s="10">
+      <c r="B60" s="10" t="str">
         <f>_xll.qlBondYield(B36,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928264971926221</v>
-      </c>
-      <c r="C60" s="10">
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
+      </c>
+      <c r="C60" s="10" t="str">
         <f>_xll.qlBondYield(C36,"actual360","CONTINUOUS","annual")</f>
-        <v>0.28928265005463161</v>
+        <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 563, in qlBondYield
+    return bond.bondYield(
+           ~~~~~~~~~~~~~~^
+        dc,
+        ^^^
+    ...&lt;3 lines&gt;...
+        max_evaluations
+        ^^^^^^^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
+    return _QuantLib.Bond_bondYield(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -7168,13 +7263,9 @@
       </c>
       <c r="B61" s="10" t="str">
         <f>_xll.qlBondPrice(B55,"clean")</f>
-        <v>欣[test_bonds.xlsx]CmsRateBond!R61C2BondPrice,A</v>
-      </c>
-      <c r="C61" s="10" t="str">
-        <f>_xll.qlBondPrice(C55,"clean")</f>
         <v>Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
     return bond.cleanPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
@@ -7183,52 +7274,31 @@
 RuntimeError: null pricing engine
 ': Expected float</v>
       </c>
+      <c r="C61" s="10" t="str">
+        <f>_xll.qlBondPrice(C55,"clean")</f>
+        <v>欣[test_bonds.xlsx]CmsRateBond!R61C3BondPrice,A</v>
+      </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B62" s="10" t="str">
         <f>_xll.qlBondYield2(B36,B61,"actual360","CONTINUOUS","annual")</f>
-        <v>0.29367879784610279</v>
-      </c>
-      <c r="C62" s="10" t="str">
+        <v>Error in arg 2 'price': Cannot convert 'Error in arg 1 'amount': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
+    return bond.cleanPrice()
+           ~~~~~~~~~~~~~~~^^
+  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
+    return _QuantLib.Bond_cleanPrice(self, *args)
+           ~~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
+RuntimeError: null pricing engine
+': Expected float': Expected cache string</v>
+      </c>
+      <c r="C62" s="10">
         <f>_xll.qlBondYield2(C36,C61,"actual360","CONTINUOUS","annual")</f>
-        <v xml:space="preserve">TypeError: TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
-  Possible C/C++ prototypes are:
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
-Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 505, in qlBondYield2
-    return bond.bondYield(
-           ~~~~~~~~~~~~~~^
-        price,
-        ^^^^^^
-    ...&lt;6 lines&gt;...
-        guess
-        ^^^^^
-    )
-    ^
-  File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25922, in bondYield
-    return _QuantLib.Bond_bondYield(self, *args)
-           ~~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^^^^^^^
-TypeError: Wrong number or type of arguments for overloaded function 'Bond_bondYield'.
-  Possible C/C++ prototypes are:
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real,Size)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency,Real)
-    Bond::yield(DayCounter const &amp;,Compounding,Frequency)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real,Size)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;,Real)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency,Date const &amp;)
-    Bond::yield(BondPrice,DayCounter const &amp;,Compounding,Frequency)
-</v>
+        <v>0.28928265005463161</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -7263,7 +7333,7 @@
         <f>_xll.qlBondSettlementValue(B36)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -7276,7 +7346,7 @@
         <f>_xll.qlBondSettlementValue(C36)</f>
         <v xml:space="preserve">RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 535, in qlBondSettlementValue
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 635, in qlBondSettlementValue
     return bond.settlementValue()
            ~~~~~~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25933, in settlementValue
@@ -7290,15 +7360,11 @@
       <c r="A66" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B66" s="10">
+      <c r="B66" s="10" t="str">
         <f>_xll.qlBondSettlementValue2(B36,B55)</f>
-        <v>159.52887538190791</v>
-      </c>
-      <c r="C66" s="10" t="str">
-        <f>_xll.qlBondSettlementValue2(C36,C55)</f>
         <v>Error in arg 2 'clean_price': Cannot convert 'RuntimeError: RuntimeError: null pricing engine
 Traceback (most recent call last):
-  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 380, in qlBondCleanPrice
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\bonds.py", line 470, in qlBondCleanPrice
     return bond.cleanPrice()
            ~~~~~~~~~~~~~~~^^
   File "C:\Users\kerst\AppData\Roaming\Python\Python314\site-packages\QuantLib\QuantLib.py", line 25908, in cleanPrice
@@ -7307,6 +7373,10 @@
 RuntimeError: null pricing engine
 ': Expected float</v>
       </c>
+      <c r="C66" s="10">
+        <f>_xll.qlBondSettlementValue2(C36,C55)</f>
+        <v>89.639709460333037</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>